<commit_message>
feat : gitignore 변경
</commit_message>
<xml_diff>
--- a/계시 환산.xlsx
+++ b/계시 환산.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gustj\Documents\GitHub\DnfHellInfo\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gustj\Documents\GitHub\dnf-hell-optimizer-react\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FACFFC88-57C6-4BFB-9CC0-B82E3AC4C22A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A63FCD4B-9D4B-4FF4-BC43-85410FAD2242}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1860" yWindow="1860" windowWidth="21600" windowHeight="11295" xr2:uid="{769C35A8-E493-4706-B4D4-CD4E84340BA2}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="107" uniqueCount="72">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="77">
   <si>
     <t>레어</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -295,6 +295,21 @@
   <si>
     <t>미광 개수</t>
     <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>레어</t>
+  </si>
+  <si>
+    <t>유니크</t>
+  </si>
+  <si>
+    <t>레전더리</t>
+  </si>
+  <si>
+    <t>무끼슬 확률</t>
+  </si>
+  <si>
+    <t>판수</t>
   </si>
 </sst>
 </file>
@@ -303,9 +318,9 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="4">
     <numFmt numFmtId="176" formatCode="0.0000%"/>
-    <numFmt numFmtId="178" formatCode="0.000%"/>
-    <numFmt numFmtId="179" formatCode="0.0000_ "/>
-    <numFmt numFmtId="180" formatCode="0_ "/>
+    <numFmt numFmtId="177" formatCode="0.000%"/>
+    <numFmt numFmtId="178" formatCode="0.0000_ "/>
+    <numFmt numFmtId="179" formatCode="0_ "/>
   </numFmts>
   <fonts count="3" x14ac:knownFonts="1">
     <font>
@@ -371,7 +386,13 @@
     <xf numFmtId="176" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="177" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="178" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
@@ -379,12 +400,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="179" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="180" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1">
-      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -720,7 +735,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{964CAE93-EE7B-4DFE-95DC-363F663B2163}">
-  <dimension ref="A1:L38"/>
+  <dimension ref="A1:L41"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="26.25" bestFit="1" customWidth="1"/>
@@ -898,19 +913,19 @@
       <c r="A7" t="s">
         <v>71</v>
       </c>
-      <c r="B7" s="9">
+      <c r="B7" s="7">
         <v>1</v>
       </c>
-      <c r="C7" s="9">
+      <c r="C7" s="7">
         <v>2</v>
       </c>
-      <c r="D7" s="9">
+      <c r="D7" s="7">
         <v>10</v>
       </c>
-      <c r="E7" s="9">
+      <c r="E7" s="7">
         <v>30</v>
       </c>
-      <c r="F7" s="9">
+      <c r="F7" s="7">
         <v>100</v>
       </c>
       <c r="G7" s="1"/>
@@ -1077,638 +1092,671 @@
       </c>
     </row>
     <row r="15" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A15" s="6" t="s">
+      <c r="B15" t="s">
+        <v>72</v>
+      </c>
+      <c r="C15" t="s">
+        <v>73</v>
+      </c>
+      <c r="D15" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="16" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
+        <v>75</v>
+      </c>
+      <c r="B16" s="1">
+        <v>0.1128</v>
+      </c>
+      <c r="C16" s="1">
+        <v>7.5899999999999995E-2</v>
+      </c>
+      <c r="D16" s="1">
+        <v>1.41E-2</v>
+      </c>
+      <c r="I16" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="I17">
+        <v>6221</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A18" s="8" t="s">
         <v>28</v>
       </c>
-      <c r="B15" s="6"/>
-      <c r="C15">
+      <c r="B18" s="8"/>
+      <c r="C18">
         <f>G4+G9</f>
         <v>12</v>
       </c>
-      <c r="E15" s="7"/>
-      <c r="F15" s="7"/>
-    </row>
-    <row r="16" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A16" s="6" t="s">
+      <c r="E18" s="9"/>
+      <c r="F18" s="9"/>
+    </row>
+    <row r="19" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A19" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="B16" s="6"/>
-      <c r="C16">
+      <c r="B19" s="8"/>
+      <c r="C19">
         <f>G4+G10</f>
         <v>14.602180152211282</v>
       </c>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A18" t="s">
+    <row r="21" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A21" t="s">
         <v>69</v>
       </c>
-      <c r="B18" t="s">
+      <c r="B21" t="s">
         <v>0</v>
       </c>
-      <c r="C18" t="s">
+      <c r="C21" t="s">
         <v>1</v>
       </c>
-      <c r="D18" t="s">
+      <c r="D21" t="s">
         <v>68</v>
       </c>
-      <c r="E18" t="s">
+      <c r="E21" t="s">
         <v>3</v>
       </c>
-      <c r="F18" t="s">
+      <c r="F21" t="s">
         <v>4</v>
       </c>
-      <c r="G18" t="s">
+      <c r="G21" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A19" s="3" t="s">
+    <row r="22" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A22" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="B19" s="8">
+      <c r="B22" s="6">
         <f>Sheet3!$B2*Sheet1!B$2</f>
         <v>3</v>
       </c>
-      <c r="C19" s="8">
+      <c r="C22" s="6">
         <f>Sheet3!$B2*Sheet1!C$2</f>
         <v>2.4000000000000004</v>
       </c>
-      <c r="D19" s="8">
+      <c r="D22" s="6">
         <f>Sheet3!$B2*Sheet1!D$2</f>
         <v>0.43199999999999994</v>
       </c>
-      <c r="E19" s="8">
+      <c r="E22" s="6">
         <f>Sheet3!$B2*Sheet1!E$2</f>
         <v>0.192</v>
       </c>
-      <c r="F19" s="8">
+      <c r="F22" s="6">
         <f>Sheet3!$B2*Sheet1!F$2</f>
         <v>1.992E-2</v>
       </c>
-      <c r="G19" s="8">
+      <c r="G22" s="6">
         <f>Sheet3!$C2*SUM($B$9:$F$9)/4</f>
         <v>27.709999999999997</v>
       </c>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A20" s="3" t="s">
+    <row r="23" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A23" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="B20" s="8">
+      <c r="B23" s="6">
         <f>Sheet3!$B3*Sheet1!B$2</f>
         <v>3</v>
       </c>
-      <c r="C20" s="8">
+      <c r="C23" s="6">
         <f>Sheet3!$B3*Sheet1!C$2</f>
         <v>2.4000000000000004</v>
       </c>
-      <c r="D20" s="8">
+      <c r="D23" s="6">
         <f>Sheet3!$B3*Sheet1!D$2</f>
         <v>0.43199999999999994</v>
       </c>
-      <c r="E20" s="8">
+      <c r="E23" s="6">
         <f>Sheet3!$B3*Sheet1!E$2</f>
         <v>0.192</v>
       </c>
-      <c r="F20" s="8">
+      <c r="F23" s="6">
         <f>Sheet3!$B3*Sheet1!F$2</f>
         <v>1.992E-2</v>
       </c>
-      <c r="G20" s="8">
+      <c r="G23" s="6">
         <f>Sheet3!$C3*SUM($B$9:$F$9)/4</f>
         <v>22.82</v>
       </c>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A21" s="3" t="s">
+    <row r="24" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A24" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="B21" s="8">
+      <c r="B24" s="6">
         <f>Sheet3!$B4*Sheet1!B$2</f>
         <v>3</v>
       </c>
-      <c r="C21" s="8">
+      <c r="C24" s="6">
         <f>Sheet3!$B4*Sheet1!C$2</f>
         <v>2.4000000000000004</v>
       </c>
-      <c r="D21" s="8">
+      <c r="D24" s="6">
         <f>Sheet3!$B4*Sheet1!D$2</f>
         <v>0.43199999999999994</v>
       </c>
-      <c r="E21" s="8">
+      <c r="E24" s="6">
         <f>Sheet3!$B4*Sheet1!E$2</f>
         <v>0.192</v>
       </c>
-      <c r="F21" s="8">
+      <c r="F24" s="6">
         <f>Sheet3!$B4*Sheet1!F$2</f>
         <v>1.992E-2</v>
       </c>
-      <c r="G21" s="8">
+      <c r="G24" s="6">
         <f>Sheet3!$C4*SUM($B$9:$F$9)/4</f>
         <v>14.669999999999998</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A22" s="3" t="s">
+    <row r="25" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A25" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="B22" s="8">
+      <c r="B25" s="6">
         <f>Sheet3!$B5*Sheet1!B$2</f>
         <v>3</v>
       </c>
-      <c r="C22" s="8">
+      <c r="C25" s="6">
         <f>Sheet3!$B5*Sheet1!C$2</f>
         <v>2.4000000000000004</v>
       </c>
-      <c r="D22" s="8">
+      <c r="D25" s="6">
         <f>Sheet3!$B5*Sheet1!D$2</f>
         <v>0.43199999999999994</v>
       </c>
-      <c r="E22" s="8">
+      <c r="E25" s="6">
         <f>Sheet3!$B5*Sheet1!E$2</f>
         <v>0.192</v>
       </c>
-      <c r="F22" s="8">
+      <c r="F25" s="6">
         <f>Sheet3!$B5*Sheet1!F$2</f>
         <v>1.992E-2</v>
       </c>
-      <c r="G22" s="8">
+      <c r="G25" s="6">
         <f>Sheet3!$C5*SUM($B$9:$F$9)/4</f>
         <v>24.45</v>
       </c>
     </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A23" s="3" t="s">
+    <row r="26" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A26" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="B23" s="8">
+      <c r="B26" s="6">
         <f>Sheet3!$B6*Sheet1!B$2</f>
         <v>3</v>
       </c>
-      <c r="C23" s="8">
+      <c r="C26" s="6">
         <f>Sheet3!$B6*Sheet1!C$2</f>
         <v>2.4000000000000004</v>
       </c>
-      <c r="D23" s="8">
+      <c r="D26" s="6">
         <f>Sheet3!$B6*Sheet1!D$2</f>
         <v>0.43199999999999994</v>
       </c>
-      <c r="E23" s="8">
+      <c r="E26" s="6">
         <f>Sheet3!$B6*Sheet1!E$2</f>
         <v>0.192</v>
       </c>
-      <c r="F23" s="8">
+      <c r="F26" s="6">
         <f>Sheet3!$B6*Sheet1!F$2</f>
         <v>1.992E-2</v>
       </c>
-      <c r="G23" s="8">
+      <c r="G26" s="6">
         <f>Sheet3!$C6*SUM($B$9:$F$9)/4</f>
         <v>19.559999999999999</v>
       </c>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A24" s="3" t="s">
+    <row r="27" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A27" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="B24" s="8">
+      <c r="B27" s="6">
         <f>Sheet3!$B7*Sheet1!B$2</f>
         <v>3</v>
       </c>
-      <c r="C24" s="8">
+      <c r="C27" s="6">
         <f>Sheet3!$B7*Sheet1!C$2</f>
         <v>2.4000000000000004</v>
       </c>
-      <c r="D24" s="8">
+      <c r="D27" s="6">
         <f>Sheet3!$B7*Sheet1!D$2</f>
         <v>0.43199999999999994</v>
       </c>
-      <c r="E24" s="8">
+      <c r="E27" s="6">
         <f>Sheet3!$B7*Sheet1!E$2</f>
         <v>0.192</v>
       </c>
-      <c r="F24" s="8">
+      <c r="F27" s="6">
         <f>Sheet3!$B7*Sheet1!F$2</f>
         <v>1.992E-2</v>
       </c>
-      <c r="G24" s="8">
+      <c r="G27" s="6">
         <f>Sheet3!$C7*SUM($B$9:$F$9)/4</f>
         <v>14.669999999999998</v>
       </c>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A25" s="3" t="s">
+    <row r="28" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A28" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="B25" s="8">
+      <c r="B28" s="6">
         <f>Sheet3!$B8*Sheet1!B$2</f>
         <v>2.75</v>
       </c>
-      <c r="C25" s="8">
+      <c r="C28" s="6">
         <f>Sheet3!$B8*Sheet1!C$2</f>
         <v>2.2000000000000002</v>
       </c>
-      <c r="D25" s="8">
+      <c r="D28" s="6">
         <f>Sheet3!$B8*Sheet1!D$2</f>
         <v>0.39599999999999996</v>
       </c>
-      <c r="E25" s="8">
+      <c r="E28" s="6">
         <f>Sheet3!$B8*Sheet1!E$2</f>
         <v>0.17599999999999999</v>
       </c>
-      <c r="F25" s="8">
+      <c r="F28" s="6">
         <f>Sheet3!$B8*Sheet1!F$2</f>
         <v>1.8259999999999998E-2</v>
       </c>
-      <c r="G25" s="8">
+      <c r="G28" s="6">
         <f>Sheet3!$C8*SUM($B$9:$F$9)/4</f>
         <v>11.41</v>
       </c>
     </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A26" s="3" t="s">
+    <row r="29" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A29" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="B26" s="8">
+      <c r="B29" s="6">
         <f>Sheet3!$B9*Sheet1!B$2</f>
         <v>2.5</v>
       </c>
-      <c r="C26" s="8">
+      <c r="C29" s="6">
         <f>Sheet3!$B9*Sheet1!C$2</f>
         <v>2</v>
       </c>
-      <c r="D26" s="8">
+      <c r="D29" s="6">
         <f>Sheet3!$B9*Sheet1!D$2</f>
         <v>0.36</v>
       </c>
-      <c r="E26" s="8">
+      <c r="E29" s="6">
         <f>Sheet3!$B9*Sheet1!E$2</f>
         <v>0.16</v>
       </c>
-      <c r="F26" s="8">
+      <c r="F29" s="6">
         <f>Sheet3!$B9*Sheet1!F$2</f>
         <v>1.66E-2</v>
       </c>
-      <c r="G26" s="8">
+      <c r="G29" s="6">
         <f>Sheet3!$C9*SUM($B$9:$F$9)/4</f>
         <v>6.52</v>
       </c>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A27" s="3" t="s">
+    <row r="30" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A30" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="B27" s="8">
+      <c r="B30" s="6">
         <f>Sheet3!$B10*Sheet1!B$2</f>
         <v>1.75</v>
       </c>
-      <c r="C27" s="8">
+      <c r="C30" s="6">
         <f>Sheet3!$B10*Sheet1!C$2</f>
         <v>1.4000000000000001</v>
       </c>
-      <c r="D27" s="8">
+      <c r="D30" s="6">
         <f>Sheet3!$B10*Sheet1!D$2</f>
         <v>0.252</v>
       </c>
-      <c r="E27" s="8">
+      <c r="E30" s="6">
         <f>Sheet3!$B10*Sheet1!E$2</f>
         <v>0.112</v>
       </c>
-      <c r="F27" s="8">
+      <c r="F30" s="6">
         <f>Sheet3!$B10*Sheet1!F$2</f>
         <v>1.162E-2</v>
       </c>
-      <c r="G27" s="8">
+      <c r="G30" s="6">
         <f>Sheet3!$C10*SUM($B$9:$F$9)/4</f>
         <v>4.8899999999999997</v>
       </c>
     </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A28" s="3" t="s">
+    <row r="31" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A31" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="B28" s="8">
+      <c r="B31" s="6">
         <f>Sheet3!$B11*Sheet1!B$2</f>
         <v>3</v>
       </c>
-      <c r="C28" s="8">
+      <c r="C31" s="6">
         <f>Sheet3!$B11*Sheet1!C$2</f>
         <v>2.4000000000000004</v>
       </c>
-      <c r="D28" s="8">
+      <c r="D31" s="6">
         <f>Sheet3!$B11*Sheet1!D$2</f>
         <v>0.43199999999999994</v>
       </c>
-      <c r="E28" s="8">
+      <c r="E31" s="6">
         <f>Sheet3!$B11*Sheet1!E$2</f>
         <v>0.192</v>
       </c>
-      <c r="F28" s="8">
+      <c r="F31" s="6">
         <f>Sheet3!$B11*Sheet1!F$2</f>
         <v>1.992E-2</v>
       </c>
-      <c r="G28" s="8">
+      <c r="G31" s="6">
         <f>Sheet3!$C11*SUM($B$9:$F$9)/4</f>
         <v>16.299999999999997</v>
       </c>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A29" s="3" t="s">
+    <row r="32" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A32" s="3" t="s">
         <v>48</v>
       </c>
-      <c r="B29" s="8">
+      <c r="B32" s="6">
         <f>Sheet3!$B12*Sheet1!B$2</f>
         <v>3</v>
       </c>
-      <c r="C29" s="8">
+      <c r="C32" s="6">
         <f>Sheet3!$B12*Sheet1!C$2</f>
         <v>2.4000000000000004</v>
       </c>
-      <c r="D29" s="8">
+      <c r="D32" s="6">
         <f>Sheet3!$B12*Sheet1!D$2</f>
         <v>0.43199999999999994</v>
       </c>
-      <c r="E29" s="8">
+      <c r="E32" s="6">
         <f>Sheet3!$B12*Sheet1!E$2</f>
         <v>0.192</v>
       </c>
-      <c r="F29" s="8">
+      <c r="F32" s="6">
         <f>Sheet3!$B12*Sheet1!F$2</f>
         <v>1.992E-2</v>
       </c>
-      <c r="G29" s="8">
+      <c r="G32" s="6">
         <f>Sheet3!$C12*SUM($B$9:$F$9)/4</f>
         <v>14.669999999999998</v>
       </c>
     </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A30" s="3" t="s">
+    <row r="33" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A33" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="B30" s="8">
+      <c r="B33" s="6">
         <f>Sheet3!$B13*Sheet1!B$2</f>
         <v>2.5</v>
       </c>
-      <c r="C30" s="8">
+      <c r="C33" s="6">
         <f>Sheet3!$B13*Sheet1!C$2</f>
         <v>2</v>
       </c>
-      <c r="D30" s="8">
+      <c r="D33" s="6">
         <f>Sheet3!$B13*Sheet1!D$2</f>
         <v>0.36</v>
       </c>
-      <c r="E30" s="8">
+      <c r="E33" s="6">
         <f>Sheet3!$B13*Sheet1!E$2</f>
         <v>0.16</v>
       </c>
-      <c r="F30" s="8">
+      <c r="F33" s="6">
         <f>Sheet3!$B13*Sheet1!F$2</f>
         <v>1.66E-2</v>
       </c>
-      <c r="G30" s="8">
+      <c r="G33" s="6">
         <f>Sheet3!$C13*SUM($B$9:$F$9)/4</f>
         <v>9.7799999999999994</v>
       </c>
     </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A31" s="3" t="s">
+    <row r="34" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A34" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="B31" s="8">
+      <c r="B34" s="6">
         <f>Sheet3!$B14*Sheet1!B$2</f>
         <v>2.25</v>
       </c>
-      <c r="C31" s="8">
+      <c r="C34" s="6">
         <f>Sheet3!$B14*Sheet1!C$2</f>
         <v>1.8</v>
       </c>
-      <c r="D31" s="8">
+      <c r="D34" s="6">
         <f>Sheet3!$B14*Sheet1!D$2</f>
         <v>0.32399999999999995</v>
       </c>
-      <c r="E31" s="8">
+      <c r="E34" s="6">
         <f>Sheet3!$B14*Sheet1!E$2</f>
         <v>0.14400000000000002</v>
       </c>
-      <c r="F31" s="8">
+      <c r="F34" s="6">
         <f>Sheet3!$B14*Sheet1!F$2</f>
         <v>1.494E-2</v>
       </c>
-      <c r="G31" s="8">
+      <c r="G34" s="6">
         <f>Sheet3!$C14*SUM($B$9:$F$9)/4</f>
         <v>8.1499999999999986</v>
       </c>
     </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A32" s="3" t="s">
+    <row r="35" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A35" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="B32" s="8">
+      <c r="B35" s="6">
         <f>Sheet3!$B15*Sheet1!B$2</f>
         <v>3</v>
       </c>
-      <c r="C32" s="8">
+      <c r="C35" s="6">
         <f>Sheet3!$B15*Sheet1!C$2</f>
         <v>2.4000000000000004</v>
       </c>
-      <c r="D32" s="8">
+      <c r="D35" s="6">
         <f>Sheet3!$B15*Sheet1!D$2</f>
         <v>0.43199999999999994</v>
       </c>
-      <c r="E32" s="8">
+      <c r="E35" s="6">
         <f>Sheet3!$B15*Sheet1!E$2</f>
         <v>0.192</v>
       </c>
-      <c r="F32" s="8">
+      <c r="F35" s="6">
         <f>Sheet3!$B15*Sheet1!F$2</f>
         <v>1.992E-2</v>
       </c>
-      <c r="G32" s="8">
+      <c r="G35" s="6">
         <f>Sheet3!$C15*SUM($B$9:$F$9)/4</f>
         <v>0</v>
       </c>
     </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A33" s="3" t="s">
+    <row r="36" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A36" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="B33" s="8">
+      <c r="B36" s="6">
         <f>Sheet3!$B16*Sheet1!B$2</f>
         <v>3</v>
       </c>
-      <c r="C33" s="8">
+      <c r="C36" s="6">
         <f>Sheet3!$B16*Sheet1!C$2</f>
         <v>2.4000000000000004</v>
       </c>
-      <c r="D33" s="8">
+      <c r="D36" s="6">
         <f>Sheet3!$B16*Sheet1!D$2</f>
         <v>0.43199999999999994</v>
       </c>
-      <c r="E33" s="8">
+      <c r="E36" s="6">
         <f>Sheet3!$B16*Sheet1!E$2</f>
         <v>0.192</v>
       </c>
-      <c r="F33" s="8">
+      <c r="F36" s="6">
         <f>Sheet3!$B16*Sheet1!F$2</f>
         <v>1.992E-2</v>
       </c>
-      <c r="G33" s="8">
+      <c r="G36" s="6">
         <f>Sheet3!$C16*SUM($B$9:$F$9)/4</f>
         <v>0</v>
       </c>
     </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A34" s="3" t="s">
+    <row r="37" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A37" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="B34" s="8">
+      <c r="B37" s="6">
         <f>Sheet3!$B17*Sheet1!B$2</f>
         <v>2</v>
       </c>
-      <c r="C34" s="8">
+      <c r="C37" s="6">
         <f>Sheet3!$B17*Sheet1!C$2</f>
         <v>1.6</v>
       </c>
-      <c r="D34" s="8">
+      <c r="D37" s="6">
         <f>Sheet3!$B17*Sheet1!D$2</f>
         <v>0.28799999999999998</v>
       </c>
-      <c r="E34" s="8">
+      <c r="E37" s="6">
         <f>Sheet3!$B17*Sheet1!E$2</f>
         <v>0.128</v>
       </c>
-      <c r="F34" s="8">
+      <c r="F37" s="6">
         <f>Sheet3!$B17*Sheet1!F$2</f>
         <v>1.328E-2</v>
       </c>
-      <c r="G34" s="8">
+      <c r="G37" s="6">
         <f>Sheet3!$C17*SUM($B$9:$F$9)/4</f>
         <v>0</v>
       </c>
     </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A35" s="3" t="s">
+    <row r="38" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A38" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="B35" s="8">
+      <c r="B38" s="6">
         <f>Sheet3!$B18*Sheet1!B$2</f>
         <v>1.75</v>
       </c>
-      <c r="C35" s="8">
+      <c r="C38" s="6">
         <f>Sheet3!$B18*Sheet1!C$2</f>
         <v>1.4000000000000001</v>
       </c>
-      <c r="D35" s="8">
+      <c r="D38" s="6">
         <f>Sheet3!$B18*Sheet1!D$2</f>
         <v>0.252</v>
       </c>
-      <c r="E35" s="8">
+      <c r="E38" s="6">
         <f>Sheet3!$B18*Sheet1!E$2</f>
         <v>0.112</v>
       </c>
-      <c r="F35" s="8">
+      <c r="F38" s="6">
         <f>Sheet3!$B18*Sheet1!F$2</f>
         <v>1.162E-2</v>
       </c>
-      <c r="G35" s="8">
+      <c r="G38" s="6">
         <f>Sheet3!$C18*SUM($B$9:$F$9)/4</f>
         <v>0</v>
       </c>
     </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A36" s="3" t="s">
+    <row r="39" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A39" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="B36" s="8">
+      <c r="B39" s="6">
         <f>Sheet3!$B19*Sheet1!B$2</f>
         <v>2</v>
       </c>
-      <c r="C36" s="8">
+      <c r="C39" s="6">
         <f>Sheet3!$B19*Sheet1!C$2</f>
         <v>1.6</v>
       </c>
-      <c r="D36" s="8">
+      <c r="D39" s="6">
         <f>Sheet3!$B19*Sheet1!D$2</f>
         <v>0.28799999999999998</v>
       </c>
-      <c r="E36" s="8">
+      <c r="E39" s="6">
         <f>Sheet3!$B19*Sheet1!E$2</f>
         <v>0.128</v>
       </c>
-      <c r="F36" s="8">
+      <c r="F39" s="6">
         <f>Sheet3!$B19*Sheet1!F$2</f>
         <v>1.328E-2</v>
       </c>
-      <c r="G36" s="8">
+      <c r="G39" s="6">
         <f>Sheet3!$C19*SUM($B$9:$F$9)/4</f>
         <v>0</v>
       </c>
     </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A37" s="3" t="s">
+    <row r="40" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A40" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="B37" s="8">
+      <c r="B40" s="6">
         <f>Sheet3!$B20*Sheet1!B$2</f>
         <v>1.25</v>
       </c>
-      <c r="C37" s="8">
+      <c r="C40" s="6">
         <f>Sheet3!$B20*Sheet1!C$2</f>
         <v>1</v>
       </c>
-      <c r="D37" s="8">
+      <c r="D40" s="6">
         <f>Sheet3!$B20*Sheet1!D$2</f>
         <v>0.18</v>
       </c>
-      <c r="E37" s="8">
+      <c r="E40" s="6">
         <f>Sheet3!$B20*Sheet1!E$2</f>
         <v>0.08</v>
       </c>
-      <c r="F37" s="8">
+      <c r="F40" s="6">
         <f>Sheet3!$B20*Sheet1!F$2</f>
         <v>8.3000000000000001E-3</v>
       </c>
-      <c r="G37" s="8">
+      <c r="G40" s="6">
         <f>Sheet3!$C20*SUM($B$9:$F$9)/4</f>
         <v>0</v>
       </c>
     </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A38" s="3" t="s">
+    <row r="41" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A41" s="3" t="s">
         <v>63</v>
       </c>
-      <c r="B38" s="8">
+      <c r="B41" s="6">
         <f>Sheet3!$B21*Sheet1!B$2</f>
         <v>3.5</v>
       </c>
-      <c r="C38" s="8">
+      <c r="C41" s="6">
         <f>Sheet3!$B21*Sheet1!C$2</f>
         <v>2.8000000000000003</v>
       </c>
-      <c r="D38" s="8">
+      <c r="D41" s="6">
         <f>Sheet3!$B21*Sheet1!D$2</f>
         <v>0.504</v>
       </c>
-      <c r="E38" s="8">
+      <c r="E41" s="6">
         <f>Sheet3!$B21*Sheet1!E$2</f>
         <v>0.224</v>
       </c>
-      <c r="F38" s="8">
+      <c r="F41" s="6">
         <f>Sheet3!$B21*Sheet1!F$2</f>
         <v>2.324E-2</v>
       </c>
-      <c r="G38" s="8">
+      <c r="G41" s="6">
         <f>Sheet3!$C21*SUM($B$9:$F$9)/4</f>
         <v>22.82</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="3">
-    <mergeCell ref="A16:B16"/>
-    <mergeCell ref="A15:B15"/>
-    <mergeCell ref="E15:F15"/>
+    <mergeCell ref="A19:B19"/>
+    <mergeCell ref="A18:B18"/>
+    <mergeCell ref="E18:F18"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
-  <conditionalFormatting sqref="B20:F38 B19">
+  <conditionalFormatting sqref="B23:F41 B22">
     <cfRule type="dataBar" priority="4">
       <dataBar>
         <cfvo type="min"/>
@@ -1722,7 +1770,7 @@
       </extLst>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C19:F19">
+  <conditionalFormatting sqref="C22:F22">
     <cfRule type="dataBar" priority="1">
       <dataBar>
         <cfvo type="min"/>
@@ -1752,7 +1800,7 @@
               <x14:axisColor rgb="FF000000"/>
             </x14:dataBar>
           </x14:cfRule>
-          <xm:sqref>B20:F38 B19</xm:sqref>
+          <xm:sqref>B23:F41 B22</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
           <x14:cfRule type="dataBar" id="{06F48B9D-DE53-4BF8-986C-3096AB01DC74}">
@@ -1765,7 +1813,7 @@
               <x14:axisColor rgb="FF000000"/>
             </x14:dataBar>
           </x14:cfRule>
-          <xm:sqref>C19:F19</xm:sqref>
+          <xm:sqref>C22:F22</xm:sqref>
         </x14:conditionalFormatting>
       </x14:conditionalFormattings>
     </ext>

</xml_diff>